<commit_message>
feat: add Supabase client with custom JWT authentication and update security audit documentation
</commit_message>
<xml_diff>
--- a/Comparativa_Auditoria_Seguridad_Final.xlsx
+++ b/Comparativa_Auditoria_Seguridad_Final.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9D2F255-DCD9-43B4-8DA3-0BACC27F444F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E6C073-777F-4916-AE2B-C407D2862ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Resumen y Diagnóstico" sheetId="1" r:id="rId1"/>
@@ -15,6 +15,10 @@
     <sheet name="⚠️ Discrepancias a Resolver" sheetId="5" r:id="rId5"/>
     <sheet name="✅ Lista Unificada Corregida" sheetId="6" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'✅ Lista Unificada Corregida'!$A$1:$J$151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'📋 Solo en DB (Faltan en Excel)'!$A$1:$J$40</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
@@ -3088,7 +3092,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3183,6 +3187,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -12752,7 +12759,7 @@
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="7" max="7" width="18" style="40" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="36" customWidth="1"/>
@@ -12809,7 +12816,7 @@
       <c r="F2" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="16" t="s">
         <v>68</v>
       </c>
       <c r="H2" s="16" t="s">
@@ -12841,7 +12848,7 @@
       <c r="F3" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="20" t="s">
         <v>71</v>
       </c>
       <c r="H3" s="20" t="s">
@@ -12873,7 +12880,7 @@
       <c r="F4" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="16" t="s">
         <v>83</v>
       </c>
       <c r="H4" s="16" t="s">
@@ -12905,7 +12912,7 @@
       <c r="F5" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="20" t="s">
         <v>91</v>
       </c>
       <c r="H5" s="20" t="s">
@@ -12937,7 +12944,7 @@
       <c r="F6" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="16" t="s">
         <v>95</v>
       </c>
       <c r="H6" s="16" t="s">
@@ -12969,7 +12976,7 @@
       <c r="F7" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="20" t="s">
         <v>110</v>
       </c>
       <c r="H7" s="20" t="s">
@@ -13001,7 +13008,7 @@
       <c r="F8" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="16" t="s">
         <v>116</v>
       </c>
       <c r="H8" s="16" t="s">
@@ -13033,7 +13040,7 @@
       <c r="F9" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="20" t="s">
         <v>139</v>
       </c>
       <c r="H9" s="20" t="s">
@@ -13065,7 +13072,7 @@
       <c r="F10" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="16" t="s">
         <v>144</v>
       </c>
       <c r="H10" s="16" t="s">
@@ -13097,7 +13104,7 @@
       <c r="F11" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="20" t="s">
         <v>148</v>
       </c>
       <c r="H11" s="20" t="s">
@@ -13129,7 +13136,7 @@
       <c r="F12" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G12" s="18" t="s">
+      <c r="G12" s="16" t="s">
         <v>151</v>
       </c>
       <c r="H12" s="16" t="s">
@@ -13161,7 +13168,7 @@
       <c r="F13" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="20" t="s">
         <v>155</v>
       </c>
       <c r="H13" s="20" t="s">
@@ -13193,7 +13200,7 @@
       <c r="F14" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G14" s="18" t="s">
+      <c r="G14" s="16" t="s">
         <v>172</v>
       </c>
       <c r="H14" s="16" t="s">
@@ -13225,7 +13232,7 @@
       <c r="F15" s="19" t="s">
         <v>176</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="G15" s="20" t="s">
         <v>177</v>
       </c>
       <c r="H15" s="20" t="s">
@@ -13257,7 +13264,7 @@
       <c r="F16" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G16" s="18" t="s">
+      <c r="G16" s="16" t="s">
         <v>180</v>
       </c>
       <c r="H16" s="16" t="s">
@@ -13289,7 +13296,7 @@
       <c r="F17" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="G17" s="19" t="s">
+      <c r="G17" s="20" t="s">
         <v>201</v>
       </c>
       <c r="H17" s="20" t="s">
@@ -13321,7 +13328,7 @@
       <c r="F18" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="G18" s="18" t="s">
+      <c r="G18" s="16" t="s">
         <v>205</v>
       </c>
       <c r="H18" s="16" t="s">
@@ -13353,7 +13360,7 @@
       <c r="F19" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="G19" s="19" t="s">
+      <c r="G19" s="20" t="s">
         <v>213</v>
       </c>
       <c r="H19" s="20" t="s">
@@ -13385,7 +13392,7 @@
       <c r="F20" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="G20" s="18" t="s">
+      <c r="G20" s="16" t="s">
         <v>220</v>
       </c>
       <c r="H20" s="16" t="s">
@@ -13417,7 +13424,7 @@
       <c r="F21" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="20" t="s">
         <v>227</v>
       </c>
       <c r="H21" s="20" t="s">
@@ -13449,7 +13456,7 @@
       <c r="F22" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="G22" s="18" t="s">
+      <c r="G22" s="16" t="s">
         <v>250</v>
       </c>
       <c r="H22" s="16" t="s">
@@ -13481,7 +13488,7 @@
       <c r="F23" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="G23" s="19" t="s">
+      <c r="G23" s="20" t="s">
         <v>257</v>
       </c>
       <c r="H23" s="20" t="s">
@@ -13513,7 +13520,7 @@
       <c r="F24" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="G24" s="18" t="s">
+      <c r="G24" s="16" t="s">
         <v>282</v>
       </c>
       <c r="H24" s="16" t="s">
@@ -13545,7 +13552,7 @@
       <c r="F25" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="G25" s="19" t="s">
+      <c r="G25" s="20" t="s">
         <v>301</v>
       </c>
       <c r="H25" s="20" t="s">
@@ -13577,7 +13584,7 @@
       <c r="F26" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="G26" s="18" t="s">
+      <c r="G26" s="16" t="s">
         <v>304</v>
       </c>
       <c r="H26" s="16" t="s">
@@ -13609,7 +13616,7 @@
       <c r="F27" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="G27" s="19" t="s">
+      <c r="G27" s="20" t="s">
         <v>311</v>
       </c>
       <c r="H27" s="20" t="s">
@@ -13641,7 +13648,7 @@
       <c r="F28" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="G28" s="18" t="s">
+      <c r="G28" s="16" t="s">
         <v>313</v>
       </c>
       <c r="H28" s="16" t="s">
@@ -13673,7 +13680,7 @@
       <c r="F29" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="G29" s="19" t="s">
+      <c r="G29" s="20" t="s">
         <v>316</v>
       </c>
       <c r="H29" s="20" t="s">
@@ -13705,7 +13712,7 @@
       <c r="F30" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="G30" s="18" t="s">
+      <c r="G30" s="16" t="s">
         <v>318</v>
       </c>
       <c r="H30" s="16" t="s">
@@ -13737,7 +13744,7 @@
       <c r="F31" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="G31" s="19" t="s">
+      <c r="G31" s="20" t="s">
         <v>320</v>
       </c>
       <c r="H31" s="20" t="s">
@@ -13769,7 +13776,7 @@
       <c r="F32" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="G32" s="18" t="s">
+      <c r="G32" s="16" t="s">
         <v>323</v>
       </c>
       <c r="H32" s="16" t="s">
@@ -13801,7 +13808,7 @@
       <c r="F33" s="19" t="s">
         <v>288</v>
       </c>
-      <c r="G33" s="19" t="s">
+      <c r="G33" s="20" t="s">
         <v>351</v>
       </c>
       <c r="H33" s="20" t="s">
@@ -13833,7 +13840,7 @@
       <c r="F34" s="18" t="s">
         <v>288</v>
       </c>
-      <c r="G34" s="18" t="s">
+      <c r="G34" s="16" t="s">
         <v>358</v>
       </c>
       <c r="H34" s="16" t="s">
@@ -13865,7 +13872,7 @@
       <c r="F35" s="19" t="s">
         <v>366</v>
       </c>
-      <c r="G35" s="19" t="s">
+      <c r="G35" s="20" t="s">
         <v>367</v>
       </c>
       <c r="H35" s="20" t="s">
@@ -13897,7 +13904,7 @@
       <c r="F36" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="G36" s="18" t="s">
+      <c r="G36" s="16" t="s">
         <v>381</v>
       </c>
       <c r="H36" s="16" t="s">
@@ -13929,7 +13936,7 @@
       <c r="F37" s="19" t="s">
         <v>288</v>
       </c>
-      <c r="G37" s="19" t="s">
+      <c r="G37" s="20" t="s">
         <v>391</v>
       </c>
       <c r="H37" s="20" t="s">
@@ -13961,7 +13968,7 @@
       <c r="F38" s="18" t="s">
         <v>288</v>
       </c>
-      <c r="G38" s="18" t="s">
+      <c r="G38" s="16" t="s">
         <v>394</v>
       </c>
       <c r="H38" s="16" t="s">
@@ -13993,7 +14000,7 @@
       <c r="F39" s="19" t="s">
         <v>288</v>
       </c>
-      <c r="G39" s="19" t="s">
+      <c r="G39" s="20" t="s">
         <v>396</v>
       </c>
       <c r="H39" s="20" t="s">
@@ -14025,7 +14032,7 @@
       <c r="F40" s="18" t="s">
         <v>288</v>
       </c>
-      <c r="G40" s="18" t="s">
+      <c r="G40" s="16" t="s">
         <v>398</v>
       </c>
       <c r="H40" s="16" t="s">
@@ -14057,7 +14064,7 @@
       <c r="F41" s="19" t="s">
         <v>288</v>
       </c>
-      <c r="G41" s="19" t="s">
+      <c r="G41" s="20" t="s">
         <v>400</v>
       </c>
       <c r="H41" s="20" t="s">
@@ -14089,7 +14096,7 @@
       <c r="F42" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="G42" s="18" t="s">
+      <c r="G42" s="16" t="s">
         <v>402</v>
       </c>
       <c r="H42" s="16" t="s">
@@ -14121,7 +14128,7 @@
       <c r="F43" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="G43" s="19" t="s">
+      <c r="G43" s="20" t="s">
         <v>404</v>
       </c>
       <c r="H43" s="20" t="s">
@@ -14153,7 +14160,7 @@
       <c r="F44" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="G44" s="18" t="s">
+      <c r="G44" s="16" t="s">
         <v>421</v>
       </c>
       <c r="H44" s="16" t="s">
@@ -14185,7 +14192,7 @@
       <c r="F45" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="G45" s="19" t="s">
+      <c r="G45" s="20" t="s">
         <v>456</v>
       </c>
       <c r="H45" s="20" t="s">
@@ -14217,7 +14224,7 @@
       <c r="F46" s="18" t="s">
         <v>200</v>
       </c>
-      <c r="G46" s="18" t="s">
+      <c r="G46" s="16" t="s">
         <v>468</v>
       </c>
       <c r="H46" s="16" t="s">
@@ -14249,7 +14256,7 @@
       <c r="F47" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="G47" s="19" t="s">
+      <c r="G47" s="20" t="s">
         <v>486</v>
       </c>
       <c r="H47" s="20" t="s">
@@ -14281,7 +14288,7 @@
       <c r="F48" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="G48" s="18" t="s">
+      <c r="G48" s="16" t="s">
         <v>509</v>
       </c>
       <c r="H48" s="16" t="s">
@@ -14313,7 +14320,7 @@
       <c r="F49" s="19" t="s">
         <v>524</v>
       </c>
-      <c r="G49" s="19" t="s">
+      <c r="G49" s="20" t="s">
         <v>525</v>
       </c>
       <c r="H49" s="20" t="s">
@@ -14345,7 +14352,7 @@
       <c r="F50" s="18" t="s">
         <v>200</v>
       </c>
-      <c r="G50" s="18" t="s">
+      <c r="G50" s="16" t="s">
         <v>527</v>
       </c>
       <c r="H50" s="16" t="s">
@@ -14377,7 +14384,7 @@
       <c r="F51" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="G51" s="19" t="s">
+      <c r="G51" s="20" t="s">
         <v>530</v>
       </c>
       <c r="H51" s="20" t="s">
@@ -14409,7 +14416,7 @@
       <c r="F52" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="G52" s="18" t="s">
+      <c r="G52" s="16" t="s">
         <v>532</v>
       </c>
       <c r="H52" s="16" t="s">
@@ -14441,7 +14448,7 @@
       <c r="F53" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="G53" s="19" t="s">
+      <c r="G53" s="20" t="s">
         <v>62</v>
       </c>
       <c r="H53" s="20" t="s">
@@ -14473,7 +14480,7 @@
       <c r="F54" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="G54" s="18" t="s">
+      <c r="G54" s="16" t="s">
         <v>541</v>
       </c>
       <c r="H54" s="16" t="s">
@@ -14505,7 +14512,7 @@
       <c r="F55" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="G55" s="19" t="s">
+      <c r="G55" s="20" t="s">
         <v>551</v>
       </c>
       <c r="H55" s="20" t="s">
@@ -14537,7 +14544,7 @@
       <c r="F56" s="18" t="s">
         <v>200</v>
       </c>
-      <c r="G56" s="18" t="s">
+      <c r="G56" s="16" t="s">
         <v>553</v>
       </c>
       <c r="H56" s="16" t="s">
@@ -14569,7 +14576,7 @@
       <c r="F57" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="G57" s="19" t="s">
+      <c r="G57" s="20" t="s">
         <v>560</v>
       </c>
       <c r="H57" s="20" t="s">
@@ -14601,7 +14608,7 @@
       <c r="F58" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="G58" s="18" t="s">
+      <c r="G58" s="16" t="s">
         <v>576</v>
       </c>
       <c r="H58" s="16" t="s">
@@ -14633,7 +14640,7 @@
       <c r="F59" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="G59" s="19" t="s">
+      <c r="G59" s="20" t="s">
         <v>579</v>
       </c>
       <c r="H59" s="20" t="s">
@@ -14665,7 +14672,7 @@
       <c r="F60" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="G60" s="18" t="s">
+      <c r="G60" s="16" t="s">
         <v>579</v>
       </c>
       <c r="H60" s="16" t="s">
@@ -14697,7 +14704,7 @@
       <c r="F61" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="G61" s="19" t="s">
+      <c r="G61" s="20" t="s">
         <v>594</v>
       </c>
       <c r="H61" s="20" t="s">
@@ -14729,7 +14736,7 @@
       <c r="F62" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="G62" s="18" t="s">
+      <c r="G62" s="16" t="s">
         <v>604</v>
       </c>
       <c r="H62" s="16" t="s">
@@ -14761,7 +14768,7 @@
       <c r="F63" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="G63" s="19" t="s">
+      <c r="G63" s="20" t="s">
         <v>594</v>
       </c>
       <c r="H63" s="20" t="s">
@@ -14783,6 +14790,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -14794,7 +14802,7 @@
     <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="42" customWidth="1"/>
+    <col min="9" max="9" width="49.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
   </cols>
   <sheetData>
@@ -14830,7 +14838,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16">
         <v>1</v>
       </c>
@@ -14894,7 +14902,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16">
         <v>3</v>
       </c>
@@ -14926,7 +14934,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="20">
         <v>4</v>
       </c>
@@ -14958,7 +14966,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16">
         <v>5</v>
       </c>
@@ -15118,7 +15126,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="20">
         <v>10</v>
       </c>
@@ -15150,7 +15158,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="16">
         <v>11</v>
       </c>
@@ -15214,7 +15222,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="16">
         <v>13</v>
       </c>
@@ -15246,7 +15254,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="20">
         <v>14</v>
       </c>
@@ -15342,7 +15350,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="16">
         <v>17</v>
       </c>
@@ -15406,7 +15414,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="16">
         <v>19</v>
       </c>
@@ -15502,7 +15510,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="20">
         <v>22</v>
       </c>
@@ -15534,7 +15542,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="16">
         <v>23</v>
       </c>
@@ -15566,7 +15574,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="20">
         <v>24</v>
       </c>
@@ -15598,7 +15606,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="16">
         <v>25</v>
       </c>
@@ -15662,7 +15670,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="16">
         <v>27</v>
       </c>
@@ -15726,7 +15734,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="16">
         <v>29</v>
       </c>
@@ -15758,7 +15766,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="20">
         <v>30</v>
       </c>
@@ -15790,7 +15798,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="16">
         <v>31</v>
       </c>
@@ -15822,7 +15830,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="20">
         <v>32</v>
       </c>
@@ -15854,7 +15862,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="16">
         <v>33</v>
       </c>
@@ -15886,7 +15894,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="20">
         <v>34</v>
       </c>
@@ -15950,7 +15958,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="20">
         <v>36</v>
       </c>
@@ -15982,7 +15990,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="16">
         <v>37</v>
       </c>
@@ -16014,7 +16022,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="20">
         <v>38</v>
       </c>
@@ -16046,7 +16054,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="16">
         <v>39</v>
       </c>
@@ -16079,7 +16087,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J40" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <autoFilter ref="A1:J40" xr:uid="{00000000-0009-0000-0000-000003000000}">
+    <filterColumn colId="7">
+      <filters>
+        <filter val="Archivado"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
@@ -17333,7 +17347,8 @@
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="8" width="14" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="17.42578125" customWidth="1"/>
     <col min="9" max="9" width="24" customWidth="1"/>
     <col min="10" max="10" width="47.5703125" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>